<commit_message>
fix: textbook (s, Q) reorder rule + publish results to a live Google Sheet
Reorder now triggers on stock position (available + on order) <= reorder point,
as in the standard (s, Q) policy; the previous "no open PO" shortcut left fast
movers stuck below their reorder point. Outputs regenerated.

Adds src/to_gsheet.py: Dashboard with live KPI formulas and two charts,
Inventory (10,000 rows, formula-driven availability and status), before/after
comparison, daily series, PO drafts, low-stock alerts, reservations, the
reconciliation report, audit log sample and a READ ME.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/05_Reconciliation.xlsx
+++ b/out/05_Reconciliation.xlsx
@@ -30,12 +30,7 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
-      <family val="2"/>
       <b val="1"/>
-      <color theme="1"/>
-      <sz val="11"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -427,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:E91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -760,23 +755,23 @@
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46227.08333333334</v>
+        <v>46226.08333333334</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>TEC-88713</t>
+          <t>GAR-52279</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>2</v>
+        <v>64</v>
       </c>
       <c r="E16" t="n">
-        <v>3</v>
+        <v>65</v>
       </c>
     </row>
     <row r="17">
@@ -790,14 +785,14 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>HEA-25746</t>
+          <t>BEA-18719</t>
         </is>
       </c>
       <c r="D17" t="n">
         <v>2</v>
       </c>
       <c r="E17" t="n">
-        <v>22</v>
+        <v>27</v>
       </c>
     </row>
     <row r="18">
@@ -811,14 +806,14 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BEA-52731</t>
+          <t>BEA-57819</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E18" t="n">
-        <v>47</v>
+        <v>63</v>
       </c>
     </row>
     <row r="19">
@@ -832,14 +827,14 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>OFF-65782</t>
+          <t>HOM-43282</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>3</v>
       </c>
       <c r="E19" t="n">
-        <v>66</v>
+        <v>26</v>
       </c>
     </row>
     <row r="20">
@@ -1084,14 +1079,14 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>OFF-83565</t>
+          <t>BEA-82490</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E31" t="n">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="32">
@@ -1105,14 +1100,14 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>HOM-88762</t>
+          <t>HOM-13038</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E32" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="33">
@@ -1126,35 +1121,35 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>OFF-16831</t>
+          <t>HOM-50891</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E33" t="n">
-        <v>106</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46235.08333333334</v>
+        <v>46234.08333333334</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>TOY-27041</t>
+          <t>HOM-45173</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>82</v>
+        <v>3</v>
       </c>
       <c r="E34" t="n">
-        <v>84</v>
+        <v>4</v>
       </c>
     </row>
     <row r="35">
@@ -1168,14 +1163,14 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>SPO-79549</t>
+          <t>GAR-90911</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
       <c r="E35" t="n">
-        <v>28</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36">
@@ -1184,40 +1179,40 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>BEA-95296</t>
+          <t>GAR-45791</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E36" t="n">
-        <v>6</v>
+        <v>13</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="n">
-        <v>46235.08333333334</v>
+        <v>46236.08333333334</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>PET-53489</t>
+          <t>HOM-32883</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E37" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
     </row>
     <row r="38">
@@ -1226,19 +1221,19 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>APP-23209</t>
+          <t>BEA-30771</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E38" t="n">
-        <v>41</v>
+        <v>29</v>
       </c>
     </row>
     <row r="39">
@@ -1252,14 +1247,14 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>APP-73163</t>
+          <t>HOM-27858</t>
         </is>
       </c>
       <c r="D39" t="n">
         <v>5</v>
       </c>
       <c r="E39" t="n">
-        <v>61</v>
+        <v>67</v>
       </c>
     </row>
     <row r="40">
@@ -1268,19 +1263,19 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>APP-25878</t>
+          <t>GAR-66898</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E40" t="n">
-        <v>34</v>
+        <v>45</v>
       </c>
     </row>
     <row r="41">
@@ -1289,66 +1284,66 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>BEA-39296</t>
+          <t>PET-77445</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E41" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46238.08333333334</v>
+        <v>46237.08333333334</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>PET-90971</t>
+          <t>SPO-45387</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>10</v>
+        <v>48</v>
       </c>
       <c r="E42" t="n">
-        <v>112</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46239.08333333334</v>
+        <v>46237.08333333334</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>PET-26696</t>
+          <t>SPO-52787</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E43" t="n">
-        <v>33</v>
+        <v>30</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46239.08333333334</v>
+        <v>46237.08333333334</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
@@ -1357,103 +1352,103 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>HOM-86902</t>
+          <t>PET-84743</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="E44" t="n">
-        <v>44</v>
+        <v>15</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46239.08333333334</v>
+        <v>46238.08333333334</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>TEC-36826</t>
+          <t>APP-41788</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E45" t="n">
-        <v>59</v>
+        <v>65</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46240.08333333334</v>
+        <v>46239.08333333334</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>PET-79411</t>
+          <t>APP-12822</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E46" t="n">
-        <v>42</v>
+        <v>40</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46241.08333333334</v>
+        <v>46239.08333333334</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>HOM-42696</t>
+          <t>TEC-88713</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="E47" t="n">
-        <v>43</v>
+        <v>34</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46241.08333333334</v>
+        <v>46239.08333333334</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>APP-94971</t>
+          <t>BEA-40347</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E48" t="n">
-        <v>21</v>
+        <v>49</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46241.08333333334</v>
+        <v>46240.08333333334</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
@@ -1462,14 +1457,14 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>TOY-88646</t>
+          <t>HOM-64715</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
       <c r="E49" t="n">
-        <v>61</v>
+        <v>68</v>
       </c>
     </row>
     <row r="50">
@@ -1483,19 +1478,19 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BEA-70069</t>
+          <t>BEA-78765</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E50" t="n">
-        <v>16</v>
+        <v>72</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46242.08333333334</v>
+        <v>46241.08333333334</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1504,19 +1499,19 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>TOY-95188</t>
+          <t>PET-96602</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E51" t="n">
-        <v>87</v>
+        <v>29</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46242.08333333334</v>
+        <v>46241.08333333334</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
@@ -1525,40 +1520,40 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>TOY-18170</t>
+          <t>GAR-94940</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>101</v>
+        <v>5</v>
       </c>
       <c r="E52" t="n">
-        <v>102</v>
+        <v>35</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46242.08333333334</v>
+        <v>46241.08333333334</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>BEA-37736</t>
+          <t>PET-51669</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>72</v>
+        <v>7</v>
       </c>
       <c r="E53" t="n">
-        <v>73</v>
+        <v>32</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46242.08333333334</v>
+        <v>46241.08333333334</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
@@ -1567,19 +1562,19 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>TOY-11404</t>
+          <t>BEA-41605</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E54" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46243.08333333334</v>
+        <v>46242.08333333334</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
@@ -1588,19 +1583,19 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>BEA-78065</t>
+          <t>GAR-71902</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E55" t="n">
-        <v>39</v>
+        <v>5</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46243.08333333334</v>
+        <v>46242.08333333334</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
@@ -1609,19 +1604,19 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>HOM-37579</t>
+          <t>GAR-52279</t>
         </is>
       </c>
       <c r="D56" t="n">
         <v>2</v>
       </c>
       <c r="E56" t="n">
-        <v>5</v>
+        <v>134</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46244.08333333334</v>
+        <v>46243.08333333334</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
@@ -1630,14 +1625,14 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>HOM-79587</t>
+          <t>OFF-57988</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>103</v>
+        <v>5</v>
       </c>
       <c r="E57" t="n">
-        <v>104</v>
+        <v>69</v>
       </c>
     </row>
     <row r="58">
@@ -1651,14 +1646,14 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>BEA-14141</t>
+          <t>OFF-90973</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E58" t="n">
-        <v>43</v>
+        <v>33</v>
       </c>
     </row>
     <row r="59">
@@ -1672,35 +1667,35 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>HOM-64108</t>
+          <t>TOY-34983</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46245.08333333334</v>
+        <v>46246.08333333334</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>TOY-34983</t>
+          <t>BEA-74255</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="E60" t="n">
-        <v>37</v>
+        <v>48</v>
       </c>
     </row>
     <row r="61">
@@ -1709,24 +1704,24 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>SPO-84339</t>
+          <t>OFF-54587</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E61" t="n">
-        <v>13</v>
+        <v>56</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46248.08333333334</v>
+        <v>46247.08333333334</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -1735,19 +1730,19 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>HOM-14594</t>
+          <t>SPO-52757</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>7</v>
+        <v>75</v>
       </c>
       <c r="E62" t="n">
-        <v>57</v>
+        <v>76</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46248.08333333334</v>
+        <v>46247.08333333334</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
@@ -1756,14 +1751,14 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>GAR-53432</t>
+          <t>TEC-37002</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E63" t="n">
-        <v>6</v>
+        <v>38</v>
       </c>
     </row>
     <row r="64">
@@ -1772,24 +1767,24 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>HOM-30892</t>
+          <t>TEC-94518</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E64" t="n">
-        <v>49</v>
+        <v>38</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46249.08333333334</v>
+        <v>46248.08333333334</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -1798,40 +1793,40 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>BEA-78576</t>
+          <t>HOM-92986</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E65" t="n">
-        <v>57</v>
+        <v>18</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46249.08333333334</v>
+        <v>46248.08333333334</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>BEA-69265</t>
+          <t>TEC-19728</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E66" t="n">
-        <v>59</v>
+        <v>63</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46250.08333333334</v>
+        <v>46248.08333333334</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -1840,82 +1835,82 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>SPO-52532</t>
+          <t>BEA-37905</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>2</v>
+        <v>75</v>
       </c>
       <c r="E67" t="n">
-        <v>20</v>
+        <v>79</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46250.08333333334</v>
+        <v>46248.08333333334</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>TOY-81809</t>
+          <t>HOM-82252</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>131</v>
+        <v>3</v>
       </c>
       <c r="E68" t="n">
-        <v>132</v>
+        <v>57</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46251.08333333334</v>
+        <v>46248.08333333334</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>HEA-78001</t>
+          <t>GAR-35325</t>
         </is>
       </c>
       <c r="D69" t="n">
         <v>4</v>
       </c>
       <c r="E69" t="n">
-        <v>44</v>
+        <v>31</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46252.08333333334</v>
+        <v>46248.08333333334</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>HOM-83945</t>
+          <t>SPO-24351</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>123</v>
+        <v>0</v>
       </c>
       <c r="E70" t="n">
-        <v>125</v>
+        <v>21</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46254.08333333334</v>
+        <v>46249.08333333334</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -1924,19 +1919,19 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>BEA-21909</t>
+          <t>SPO-61232</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>44</v>
+        <v>5</v>
       </c>
       <c r="E71" t="n">
-        <v>45</v>
+        <v>6</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46254.08333333334</v>
+        <v>46250.08333333334</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
@@ -1945,287 +1940,413 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>APP-83641</t>
+          <t>BEA-70565</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E72" t="n">
-        <v>25</v>
+        <v>32</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46254.08333333334</v>
+        <v>46251.08333333334</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>PET-17098</t>
+          <t>TOY-85161</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>2</v>
+        <v>148</v>
       </c>
       <c r="E73" t="n">
-        <v>4</v>
+        <v>149</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46256.08333333334</v>
+        <v>46251.08333333334</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>BEA-40241</t>
+          <t>SPO-26486</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="E74" t="n">
-        <v>21</v>
+        <v>30</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46257.08333333334</v>
+        <v>46252.08333333334</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>SPO-91980</t>
+          <t>SPO-37801</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E75" t="n">
-        <v>6</v>
+        <v>35</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46257.08333333334</v>
+        <v>46252.08333333334</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>HEA-71592</t>
+          <t>SPO-22387</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E76" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46260.08333333334</v>
+        <v>46253.08333333334</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>APP-83748</t>
+          <t>SPO-73654</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="E77" t="n">
-        <v>57</v>
+        <v>17</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46260.08333333334</v>
+        <v>46254.08333333334</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>SPO-95544</t>
+          <t>TOY-40316</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>17</v>
+        <v>1</v>
       </c>
       <c r="E78" t="n">
-        <v>18</v>
+        <v>68</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46261.08333333334</v>
+        <v>46254.08333333334</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>GAR-26841</t>
+          <t>BEA-96573</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E79" t="n">
-        <v>47</v>
+        <v>9</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46261.08333333334</v>
+        <v>46254.08333333334</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>APP-49051</t>
+          <t>PET-58127</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="E80" t="n">
-        <v>14</v>
+        <v>24</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46261.08333333334</v>
+        <v>46255.08333333334</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>PET-80884</t>
+          <t>APP-29988</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>30</v>
+        <v>1</v>
       </c>
       <c r="E81" t="n">
-        <v>31</v>
+        <v>46</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="n">
-        <v>46261.08333333334</v>
+        <v>46256.08333333334</v>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>TOY-41164</t>
+          <t>OFF-89997</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E82" t="n">
-        <v>10</v>
+        <v>59</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="n">
-        <v>46261.08333333334</v>
+        <v>46257.08333333334</v>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>HOM-65012</t>
+          <t>PET-90647</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>6</v>
+        <v>181</v>
       </c>
       <c r="E83" t="n">
-        <v>43</v>
+        <v>182</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="n">
-        <v>46261.08333333334</v>
+        <v>46257.08333333334</v>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>SPO-81299</t>
+          <t>TOY-39114</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E84" t="n">
-        <v>74</v>
+        <v>40</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="n">
-        <v>46263.08333333334</v>
+        <v>46259.08333333334</v>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>APP-51438</t>
+          <t>SPO-44410</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>0</v>
+        <v>9</v>
       </c>
       <c r="E85" t="n">
-        <v>31</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="n">
+        <v>46260.08333333334</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>HOM-88901</t>
+        </is>
+      </c>
+      <c r="D86" t="n">
+        <v>1</v>
+      </c>
+      <c r="E86" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="2" t="n">
+        <v>46260.08333333334</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>WEB</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>HOM-87146</t>
+        </is>
+      </c>
+      <c r="D87" t="n">
+        <v>5</v>
+      </c>
+      <c r="E87" t="n">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="n">
+        <v>46260.08333333334</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>MKA</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>BEA-22481</t>
+        </is>
+      </c>
+      <c r="D88" t="n">
+        <v>3</v>
+      </c>
+      <c r="E88" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="2" t="n">
+        <v>46260.08333333334</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>MKA</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>APP-91104</t>
+        </is>
+      </c>
+      <c r="D89" t="n">
+        <v>2</v>
+      </c>
+      <c r="E89" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="n">
+        <v>46261.08333333334</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>MKA</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>HOM-24885</t>
+        </is>
+      </c>
+      <c r="D90" t="n">
+        <v>61</v>
+      </c>
+      <c r="E90" t="n">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="2" t="n">
+        <v>46261.08333333334</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>MKA</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>TOY-58894</t>
+        </is>
+      </c>
+      <c r="D91" t="n">
+        <v>7</v>
+      </c>
+      <c r="E91" t="n">
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix: fair before/after and honest claims after adversarial review
- both strategies now share webhook de-duplication; the only difference
  measured is how stock reaches the channels (oversells 257 -> 239 daily)
- stress run: every channel push 20x slower -> reported, not hidden
- alert cooldown bug: a crossing held back by the cooldown now fires once
  the cooldown ends (+ test)
- invariant check uses what channels SHOW, not what they are offered
- removed strawman comparisons (level pings, full-catalogue pushes) and the
  "more units sold" claim; channel APIs stated as simulated everywhere
- publish buffer off by default (measured: no effect on oversells)
- sheet_snapshots takes a spreadsheet id; requirements complete

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/05_Reconciliation.xlsx
+++ b/out/05_Reconciliation.xlsx
@@ -422,7 +422,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E91"/>
+  <dimension ref="A1:E81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="21" customWidth="1" min="1" max="1"/>
@@ -545,7 +545,7 @@
     </row>
     <row r="6">
       <c r="A6" s="2" t="n">
-        <v>46214.08333333334</v>
+        <v>46216.08333333334</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -554,133 +554,133 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>GAR-19772</t>
+          <t>PET-94607</t>
         </is>
       </c>
       <c r="D6" t="n">
-        <v>20</v>
+        <v>6</v>
       </c>
       <c r="E6" t="n">
-        <v>21</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="n">
-        <v>46216.08333333334</v>
+        <v>46217.08333333334</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>APP-50624</t>
+          <t>OFF-37179</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>112</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="n">
-        <v>46217.08333333334</v>
+        <v>46220.08333333334</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>OFF-37179</t>
+          <t>APP-78550</t>
         </is>
       </c>
       <c r="D8" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E8" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="n">
-        <v>46217.08333333334</v>
+        <v>46220.08333333334</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>OFF-13444</t>
+          <t>APP-29988</t>
         </is>
       </c>
       <c r="D9" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E9" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="n">
-        <v>46217.08333333334</v>
+        <v>46221.08333333334</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>OFF-41623</t>
+          <t>HOM-74246</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E10" t="n">
-        <v>33</v>
+        <v>16</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="n">
-        <v>46218.08333333334</v>
+        <v>46222.08333333334</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>BEA-91207</t>
+          <t>BEA-19113</t>
         </is>
       </c>
       <c r="D11" t="n">
-        <v>92</v>
+        <v>187</v>
       </c>
       <c r="E11" t="n">
-        <v>93</v>
+        <v>188</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n">
-        <v>46219.08333333334</v>
+        <v>46223.08333333334</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>TEC-78735</t>
+          <t>OFF-74309</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -692,91 +692,91 @@
     </row>
     <row r="13">
       <c r="A13" s="2" t="n">
-        <v>46221.08333333334</v>
+        <v>46224.08333333334</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>TEC-84299</t>
+          <t>TEC-32018</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>51</v>
+        <v>15</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="n">
-        <v>46224.08333333334</v>
+        <v>46226.08333333334</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>GAR-41242</t>
+          <t>BEA-91155</t>
         </is>
       </c>
       <c r="D14" t="n">
-        <v>27</v>
+        <v>5</v>
       </c>
       <c r="E14" t="n">
-        <v>28</v>
+        <v>39</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="n">
-        <v>46224.08333333334</v>
+        <v>46227.08333333334</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>GAR-60383</t>
+          <t>HOM-15844</t>
         </is>
       </c>
       <c r="D15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="E15" t="n">
-        <v>48</v>
+        <v>6</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n">
-        <v>46226.08333333334</v>
+        <v>46227.08333333334</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>GAR-52279</t>
+          <t>HOM-85251</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>64</v>
+        <v>8</v>
       </c>
       <c r="E16" t="n">
-        <v>65</v>
+        <v>41</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="n">
-        <v>46227.08333333334</v>
+        <v>46228.08333333334</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
@@ -785,19 +785,19 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BEA-18719</t>
+          <t>BEA-92564</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E17" t="n">
-        <v>27</v>
+        <v>41</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="n">
-        <v>46228.08333333334</v>
+        <v>46229.08333333334</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
@@ -806,35 +806,35 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>BEA-57819</t>
+          <t>TEC-93923</t>
         </is>
       </c>
       <c r="D18" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E18" t="n">
-        <v>63</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="n">
-        <v>46228.08333333334</v>
+        <v>46229.08333333334</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>HOM-43282</t>
+          <t>SPO-48666</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E19" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20">
@@ -848,14 +848,14 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>TOY-85684</t>
+          <t>BEA-42423</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>10</v>
+        <v>4</v>
       </c>
       <c r="E20" t="n">
-        <v>111</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21">
@@ -864,19 +864,19 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>TEC-90715</t>
+          <t>HOM-98411</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E21" t="n">
-        <v>35</v>
+        <v>22</v>
       </c>
     </row>
     <row r="22">
@@ -885,24 +885,24 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>APP-88180</t>
+          <t>HOM-75685</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="E22" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="n">
-        <v>46229.08333333334</v>
+        <v>46231.08333333334</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
@@ -911,40 +911,40 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>BEA-50911</t>
+          <t>HOM-64576</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="E23" t="n">
-        <v>13</v>
+        <v>112</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="n">
-        <v>46229.08333333334</v>
+        <v>46231.08333333334</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>HOM-96618</t>
+          <t>TEC-50829</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="E24" t="n">
-        <v>46</v>
+        <v>26</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="n">
-        <v>46231.08333333334</v>
+        <v>46232.08333333334</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
@@ -953,19 +953,19 @@
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>GAR-57800</t>
+          <t>BEA-26279</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E25" t="n">
-        <v>7</v>
+        <v>43</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="n">
-        <v>46231.08333333334</v>
+        <v>46232.08333333334</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
@@ -974,19 +974,19 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>SPO-96002</t>
+          <t>SPO-15808</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E26" t="n">
-        <v>32</v>
+        <v>5</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="n">
-        <v>46231.08333333334</v>
+        <v>46232.08333333334</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
@@ -995,14 +995,14 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>APP-15986</t>
+          <t>HOM-15210</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E27" t="n">
-        <v>10</v>
+        <v>40</v>
       </c>
     </row>
     <row r="28">
@@ -1011,45 +1011,45 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>BEA-65925</t>
+          <t>BEA-87032</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="E28" t="n">
-        <v>103</v>
+        <v>72</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="n">
-        <v>46232.08333333334</v>
+        <v>46233.08333333334</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>HOM-75591</t>
+          <t>PET-22306</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>34</v>
+        <v>19</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="n">
-        <v>46232.08333333334</v>
+        <v>46233.08333333334</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
@@ -1058,40 +1058,40 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>TEC-33011</t>
+          <t>TEC-44507</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>6</v>
+        <v>11</v>
       </c>
       <c r="E30" t="n">
-        <v>36</v>
+        <v>12</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="n">
-        <v>46233.08333333334</v>
+        <v>46234.08333333334</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>BEA-82490</t>
+          <t>TEC-69918</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>51</v>
+        <v>142</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="n">
-        <v>46233.08333333334</v>
+        <v>46235.08333333334</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
@@ -1100,40 +1100,40 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>HOM-13038</t>
+          <t>SPO-38242</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>2</v>
+        <v>12</v>
       </c>
       <c r="E32" t="n">
-        <v>36</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="n">
-        <v>46234.08333333334</v>
+        <v>46235.08333333334</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>HOM-50891</t>
+          <t>HOM-87808</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E33" t="n">
-        <v>29</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="n">
-        <v>46234.08333333334</v>
+        <v>46235.08333333334</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
@@ -1142,14 +1142,14 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>HOM-45173</t>
+          <t>TOY-18125</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E34" t="n">
-        <v>4</v>
+        <v>22</v>
       </c>
     </row>
     <row r="35">
@@ -1158,19 +1158,19 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>GAR-90911</t>
+          <t>TOY-11254</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E35" t="n">
-        <v>8</v>
+        <v>123</v>
       </c>
     </row>
     <row r="36">
@@ -1184,14 +1184,14 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>GAR-45791</t>
+          <t>TEC-21979</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E36" t="n">
-        <v>13</v>
+        <v>47</v>
       </c>
     </row>
     <row r="37">
@@ -1205,14 +1205,14 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>HOM-32883</t>
+          <t>PET-64678</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>29</v>
+        <v>22</v>
       </c>
     </row>
     <row r="38">
@@ -1226,14 +1226,14 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>BEA-30771</t>
+          <t>HOM-70624</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E38" t="n">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
     <row r="39">
@@ -1247,61 +1247,61 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>HOM-27858</t>
+          <t>HOM-33205</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E39" t="n">
-        <v>67</v>
+        <v>27</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="n">
-        <v>46236.08333333334</v>
+        <v>46238.08333333334</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>GAR-66898</t>
+          <t>APP-45687</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>4</v>
+        <v>12</v>
       </c>
       <c r="E40" t="n">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="n">
-        <v>46237.08333333334</v>
+        <v>46239.08333333334</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>PET-77445</t>
+          <t>TEC-90179</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="E41" t="n">
-        <v>5</v>
+        <v>61</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="n">
-        <v>46237.08333333334</v>
+        <v>46239.08333333334</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
@@ -1310,19 +1310,19 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>SPO-45387</t>
+          <t>TEC-85168</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>48</v>
+        <v>5</v>
       </c>
       <c r="E42" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="n">
-        <v>46237.08333333334</v>
+        <v>46239.08333333334</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
@@ -1331,166 +1331,166 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>SPO-52787</t>
+          <t>TOY-48773</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E43" t="n">
-        <v>30</v>
+        <v>68</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="n">
-        <v>46237.08333333334</v>
+        <v>46240.08333333334</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>PET-84743</t>
+          <t>PET-80884</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="E44" t="n">
-        <v>15</v>
+        <v>37</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="n">
-        <v>46238.08333333334</v>
+        <v>46240.08333333334</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>APP-41788</t>
+          <t>HOM-95406</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E45" t="n">
-        <v>65</v>
+        <v>36</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="n">
-        <v>46239.08333333334</v>
+        <v>46241.08333333334</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>APP-12822</t>
+          <t>PET-51647</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>9</v>
+        <v>4</v>
       </c>
       <c r="E46" t="n">
-        <v>40</v>
+        <v>36</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="n">
-        <v>46239.08333333334</v>
+        <v>46241.08333333334</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>TEC-88713</t>
+          <t>TOY-94761</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E47" t="n">
-        <v>34</v>
+        <v>31</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="n">
-        <v>46239.08333333334</v>
+        <v>46241.08333333334</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>BEA-40347</t>
+          <t>TOY-19533</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
       <c r="E48" t="n">
-        <v>49</v>
+        <v>30</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="n">
-        <v>46240.08333333334</v>
+        <v>46241.08333333334</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>HOM-64715</t>
+          <t>BEA-99017</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="E49" t="n">
-        <v>68</v>
+        <v>20</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="n">
-        <v>46241.08333333334</v>
+        <v>46243.08333333334</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BEA-78765</t>
+          <t>HEA-78679</t>
         </is>
       </c>
       <c r="D50" t="n">
         <v>6</v>
       </c>
       <c r="E50" t="n">
-        <v>72</v>
+        <v>33</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="n">
-        <v>46241.08333333334</v>
+        <v>46245.08333333334</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
@@ -1499,40 +1499,40 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>PET-96602</t>
+          <t>HOM-21081</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E51" t="n">
-        <v>29</v>
+        <v>101</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="n">
-        <v>46241.08333333334</v>
+        <v>46245.08333333334</v>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>GAR-94940</t>
+          <t>OFF-36207</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E52" t="n">
-        <v>35</v>
+        <v>24</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="n">
-        <v>46241.08333333334</v>
+        <v>46246.08333333334</v>
       </c>
       <c r="B53" t="inlineStr">
         <is>
@@ -1541,103 +1541,103 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>PET-51669</t>
+          <t>BEA-26849</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E53" t="n">
-        <v>32</v>
+        <v>39</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="n">
-        <v>46241.08333333334</v>
+        <v>46246.08333333334</v>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>BEA-41605</t>
+          <t>TEC-64512</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E54" t="n">
-        <v>23</v>
+        <v>53</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="n">
-        <v>46242.08333333334</v>
+        <v>46247.08333333334</v>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>GAR-71902</t>
+          <t>SPO-40478</t>
         </is>
       </c>
       <c r="D55" t="n">
         <v>4</v>
       </c>
       <c r="E55" t="n">
-        <v>5</v>
+        <v>44</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="n">
-        <v>46242.08333333334</v>
+        <v>46248.08333333334</v>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>GAR-52279</t>
+          <t>HOM-14594</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E56" t="n">
-        <v>134</v>
+        <v>57</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="n">
-        <v>46243.08333333334</v>
+        <v>46248.08333333334</v>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>OFF-57988</t>
+          <t>HOM-19630</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E57" t="n">
-        <v>69</v>
+        <v>26</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="n">
-        <v>46245.08333333334</v>
+        <v>46248.08333333334</v>
       </c>
       <c r="B58" t="inlineStr">
         <is>
@@ -1646,19 +1646,19 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>OFF-90973</t>
+          <t>APP-25679</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E58" t="n">
-        <v>33</v>
+        <v>46</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="2" t="n">
-        <v>46245.08333333334</v>
+        <v>46248.08333333334</v>
       </c>
       <c r="B59" t="inlineStr">
         <is>
@@ -1667,61 +1667,61 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>TOY-34983</t>
+          <t>HOM-48378</t>
         </is>
       </c>
       <c r="D59" t="n">
         <v>0</v>
       </c>
       <c r="E59" t="n">
-        <v>37</v>
+        <v>20</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="n">
-        <v>46246.08333333334</v>
+        <v>46248.08333333334</v>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>BEA-74255</t>
+          <t>HOM-31461</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E60" t="n">
-        <v>48</v>
+        <v>168</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="n">
-        <v>46246.08333333334</v>
+        <v>46249.08333333334</v>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>OFF-54587</t>
+          <t>HOM-37571</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E61" t="n">
-        <v>56</v>
+        <v>6</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="n">
-        <v>46247.08333333334</v>
+        <v>46249.08333333334</v>
       </c>
       <c r="B62" t="inlineStr">
         <is>
@@ -1730,61 +1730,61 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>SPO-52757</t>
+          <t>HOM-33941</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>75</v>
+        <v>1</v>
       </c>
       <c r="E62" t="n">
-        <v>76</v>
+        <v>21</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="n">
-        <v>46247.08333333334</v>
+        <v>46250.08333333334</v>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>TEC-37002</t>
+          <t>BEA-81500</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E63" t="n">
-        <v>38</v>
+        <v>14</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="n">
-        <v>46248.08333333334</v>
+        <v>46251.08333333334</v>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>TEC-94518</t>
+          <t>BEA-75558</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E64" t="n">
-        <v>38</v>
+        <v>55</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="n">
-        <v>46248.08333333334</v>
+        <v>46252.08333333334</v>
       </c>
       <c r="B65" t="inlineStr">
         <is>
@@ -1793,19 +1793,19 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>HOM-92986</t>
+          <t>TEC-11765</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="E65" t="n">
-        <v>18</v>
+        <v>40</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="n">
-        <v>46248.08333333334</v>
+        <v>46252.08333333334</v>
       </c>
       <c r="B66" t="inlineStr">
         <is>
@@ -1814,19 +1814,19 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>TEC-19728</t>
+          <t>PET-97502</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E66" t="n">
-        <v>63</v>
+        <v>57</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="n">
-        <v>46248.08333333334</v>
+        <v>46254.08333333334</v>
       </c>
       <c r="B67" t="inlineStr">
         <is>
@@ -1835,19 +1835,19 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>BEA-37905</t>
+          <t>HEA-85181</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>75</v>
+        <v>2</v>
       </c>
       <c r="E67" t="n">
-        <v>79</v>
+        <v>3</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="2" t="n">
-        <v>46248.08333333334</v>
+        <v>46254.08333333334</v>
       </c>
       <c r="B68" t="inlineStr">
         <is>
@@ -1856,19 +1856,19 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>HOM-82252</t>
+          <t>SPO-72301</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E68" t="n">
-        <v>57</v>
+        <v>12</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="n">
-        <v>46248.08333333334</v>
+        <v>46254.08333333334</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
@@ -1877,19 +1877,19 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>GAR-35325</t>
+          <t>TOY-78616</t>
         </is>
       </c>
       <c r="D69" t="n">
         <v>4</v>
       </c>
       <c r="E69" t="n">
-        <v>31</v>
+        <v>6</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="2" t="n">
-        <v>46248.08333333334</v>
+        <v>46254.08333333334</v>
       </c>
       <c r="B70" t="inlineStr">
         <is>
@@ -1898,19 +1898,19 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>SPO-24351</t>
+          <t>SPO-24220</t>
         </is>
       </c>
       <c r="D70" t="n">
         <v>0</v>
       </c>
       <c r="E70" t="n">
-        <v>21</v>
+        <v>12</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="n">
-        <v>46249.08333333334</v>
+        <v>46255.08333333334</v>
       </c>
       <c r="B71" t="inlineStr">
         <is>
@@ -1919,40 +1919,40 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SPO-61232</t>
+          <t>BEA-95514</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>5</v>
+        <v>151</v>
       </c>
       <c r="E71" t="n">
-        <v>6</v>
+        <v>152</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="n">
-        <v>46250.08333333334</v>
+        <v>46255.08333333334</v>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>BEA-70565</t>
+          <t>HOM-14271</t>
         </is>
       </c>
       <c r="D72" t="n">
         <v>1</v>
       </c>
       <c r="E72" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="n">
-        <v>46251.08333333334</v>
+        <v>46257.08333333334</v>
       </c>
       <c r="B73" t="inlineStr">
         <is>
@@ -1961,19 +1961,19 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>TOY-85161</t>
+          <t>HOM-99467</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>148</v>
+        <v>0</v>
       </c>
       <c r="E73" t="n">
-        <v>149</v>
+        <v>37</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="2" t="n">
-        <v>46251.08333333334</v>
+        <v>46259.08333333334</v>
       </c>
       <c r="B74" t="inlineStr">
         <is>
@@ -1982,61 +1982,61 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>SPO-26486</t>
+          <t>HEA-10839</t>
         </is>
       </c>
       <c r="D74" t="n">
+        <v>4</v>
+      </c>
+      <c r="E74" t="n">
         <v>29</v>
-      </c>
-      <c r="E74" t="n">
-        <v>30</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="n">
-        <v>46252.08333333334</v>
+        <v>46260.08333333334</v>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>SPO-37801</t>
+          <t>HOM-60806</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>4</v>
+        <v>15</v>
       </c>
       <c r="E75" t="n">
-        <v>35</v>
+        <v>79</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="n">
-        <v>46252.08333333334</v>
+        <v>46260.08333333334</v>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>WEB</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>SPO-22387</t>
+          <t>TEC-97784</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>3</v>
+        <v>27</v>
       </c>
       <c r="E76" t="n">
-        <v>32</v>
+        <v>29</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="n">
-        <v>46253.08333333334</v>
+        <v>46260.08333333334</v>
       </c>
       <c r="B77" t="inlineStr">
         <is>
@@ -2045,82 +2045,82 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>SPO-73654</t>
+          <t>HOM-64788</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E77" t="n">
-        <v>17</v>
+        <v>27</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="n">
-        <v>46254.08333333334</v>
+        <v>46260.08333333334</v>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>WEB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>TOY-40316</t>
+          <t>BEA-62879</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E78" t="n">
-        <v>68</v>
+        <v>40</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="n">
-        <v>46254.08333333334</v>
+        <v>46260.08333333334</v>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>MKA</t>
+          <t>MKB</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>BEA-96573</t>
+          <t>GAR-28241</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>8</v>
+        <v>37</v>
       </c>
       <c r="E79" t="n">
-        <v>9</v>
+        <v>38</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="n">
-        <v>46254.08333333334</v>
+        <v>46261.08333333334</v>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>MKB</t>
+          <t>MKA</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>PET-58127</t>
+          <t>PET-14922</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E80" t="n">
-        <v>24</v>
+        <v>38</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="n">
-        <v>46255.08333333334</v>
+        <v>46262.08333333334</v>
       </c>
       <c r="B81" t="inlineStr">
         <is>
@@ -2129,224 +2129,14 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>APP-29988</t>
+          <t>BEA-13135</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>1</v>
+        <v>122</v>
       </c>
       <c r="E81" t="n">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="82">
-      <c r="A82" s="2" t="n">
-        <v>46256.08333333334</v>
-      </c>
-      <c r="B82" t="inlineStr">
-        <is>
-          <t>WEB</t>
-        </is>
-      </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>OFF-89997</t>
-        </is>
-      </c>
-      <c r="D82" t="n">
-        <v>7</v>
-      </c>
-      <c r="E82" t="n">
-        <v>59</v>
-      </c>
-    </row>
-    <row r="83">
-      <c r="A83" s="2" t="n">
-        <v>46257.08333333334</v>
-      </c>
-      <c r="B83" t="inlineStr">
-        <is>
-          <t>WEB</t>
-        </is>
-      </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>PET-90647</t>
-        </is>
-      </c>
-      <c r="D83" t="n">
-        <v>181</v>
-      </c>
-      <c r="E83" t="n">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" s="2" t="n">
-        <v>46257.08333333334</v>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>MKA</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>TOY-39114</t>
-        </is>
-      </c>
-      <c r="D84" t="n">
-        <v>3</v>
-      </c>
-      <c r="E84" t="n">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="85">
-      <c r="A85" s="2" t="n">
-        <v>46259.08333333334</v>
-      </c>
-      <c r="B85" t="inlineStr">
-        <is>
-          <t>MKB</t>
-        </is>
-      </c>
-      <c r="C85" t="inlineStr">
-        <is>
-          <t>SPO-44410</t>
-        </is>
-      </c>
-      <c r="D85" t="n">
-        <v>9</v>
-      </c>
-      <c r="E85" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="86">
-      <c r="A86" s="2" t="n">
-        <v>46260.08333333334</v>
-      </c>
-      <c r="B86" t="inlineStr">
-        <is>
-          <t>WEB</t>
-        </is>
-      </c>
-      <c r="C86" t="inlineStr">
-        <is>
-          <t>HOM-88901</t>
-        </is>
-      </c>
-      <c r="D86" t="n">
-        <v>1</v>
-      </c>
-      <c r="E86" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="87">
-      <c r="A87" s="2" t="n">
-        <v>46260.08333333334</v>
-      </c>
-      <c r="B87" t="inlineStr">
-        <is>
-          <t>WEB</t>
-        </is>
-      </c>
-      <c r="C87" t="inlineStr">
-        <is>
-          <t>HOM-87146</t>
-        </is>
-      </c>
-      <c r="D87" t="n">
-        <v>5</v>
-      </c>
-      <c r="E87" t="n">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="88">
-      <c r="A88" s="2" t="n">
-        <v>46260.08333333334</v>
-      </c>
-      <c r="B88" t="inlineStr">
-        <is>
-          <t>MKA</t>
-        </is>
-      </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>BEA-22481</t>
-        </is>
-      </c>
-      <c r="D88" t="n">
-        <v>3</v>
-      </c>
-      <c r="E88" t="n">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="89">
-      <c r="A89" s="2" t="n">
-        <v>46260.08333333334</v>
-      </c>
-      <c r="B89" t="inlineStr">
-        <is>
-          <t>MKA</t>
-        </is>
-      </c>
-      <c r="C89" t="inlineStr">
-        <is>
-          <t>APP-91104</t>
-        </is>
-      </c>
-      <c r="D89" t="n">
-        <v>2</v>
-      </c>
-      <c r="E89" t="n">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="90">
-      <c r="A90" s="2" t="n">
-        <v>46261.08333333334</v>
-      </c>
-      <c r="B90" t="inlineStr">
-        <is>
-          <t>MKA</t>
-        </is>
-      </c>
-      <c r="C90" t="inlineStr">
-        <is>
-          <t>HOM-24885</t>
-        </is>
-      </c>
-      <c r="D90" t="n">
-        <v>61</v>
-      </c>
-      <c r="E90" t="n">
-        <v>63</v>
-      </c>
-    </row>
-    <row r="91">
-      <c r="A91" s="2" t="n">
-        <v>46261.08333333334</v>
-      </c>
-      <c r="B91" t="inlineStr">
-        <is>
-          <t>MKA</t>
-        </is>
-      </c>
-      <c r="C91" t="inlineStr">
-        <is>
-          <t>TOY-58894</t>
-        </is>
-      </c>
-      <c r="D91" t="n">
-        <v>7</v>
-      </c>
-      <c r="E91" t="n">
-        <v>63</v>
+        <v>123</v>
       </c>
     </row>
   </sheetData>
@@ -2363,7 +2153,7 @@
   <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="8" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
@@ -2430,7 +2220,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>no channel offered more than available</t>
+          <t>no channel shows more than available (end of run)</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">

</xml_diff>